<commit_message>
fix(ssot): eliminate company name truncation, expand autofilter coverage to full tables, and deepen data validations
</commit_message>
<xml_diff>
--- a/Master_Internship_Tracker_2027_SSOT.xlsx
+++ b/Master_Internship_Tracker_2027_SSOT.xlsx
@@ -18,13 +18,13 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'0.CEO_Dashboard'!$B$11:$G$18</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'1.UK_Top_Targets'!$A$1:$K$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'1.UK_Top_Targets'!$A$1:$L$21</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'2.UK_Tech_Quant_Finance'!$A$1:$I$685</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'3.KR_타임라인_우선순위'!$A$1:$K$56</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'4.KR_Tech_BCI'!$A$2:$I$41</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'5.KR_전략_대기업_금융'!$A$2:$I$30</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'6.Global_BCI_Map'!$A$1:$E$29</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'7.BCI_Research_DB'!$A$1:$F$85</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'7.BCI_Research_DB'!$A$1:$K$85</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1826,16 +1826,16 @@
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="36" customWidth="1" min="3" max="3"/>
-    <col width="52" customWidth="1" min="4" max="4"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="62" customWidth="1" min="4" max="4"/>
     <col width="28" customWidth="1" min="5" max="5"/>
-    <col width="28" customWidth="1" min="6" max="6"/>
+    <col width="32" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="36" customWidth="1" min="8" max="8"/>
-    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="42" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="9" max="9"/>
     <col width="18" customWidth="1" min="10" max="10"/>
     <col width="22" customWidth="1" min="11" max="11"/>
-    <col width="65" customWidth="1" min="12" max="12"/>
+    <col width="75" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -3112,7 +3112,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K21"/>
+  <autoFilter ref="A1:L21"/>
   <dataValidations count="2">
     <dataValidation sqref="J2:J21" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"To-Apply (L1),To-Apply (L2),Applied,Interview,Offer,Rejected,Saved"</formula1>
@@ -3159,12 +3159,12 @@
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="36" customWidth="1" min="3" max="3"/>
-    <col width="62" customWidth="1" min="4" max="4"/>
-    <col width="42" customWidth="1" min="5" max="5"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
+    <col width="82" customWidth="1" min="4" max="4"/>
+    <col width="55" customWidth="1" min="5" max="5"/>
     <col width="26" customWidth="1" min="6" max="6"/>
     <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="26" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
     <col width="20" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
@@ -31511,17 +31511,17 @@
   <dimension ref="A1:K56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
     <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="46" customWidth="1" min="3" max="3"/>
-    <col width="32" customWidth="1" min="4" max="4"/>
-    <col width="26" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
-    <col width="40" customWidth="1" min="7" max="7"/>
-    <col width="48" customWidth="1" min="8" max="8"/>
+    <col width="65" customWidth="1" min="3" max="3"/>
+    <col width="46" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
+    <col width="42" customWidth="1" min="7" max="7"/>
+    <col width="50" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
     <col width="18" customWidth="1" min="10" max="10"/>
-    <col width="32" customWidth="1" min="11" max="11"/>
+    <col width="34" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -34787,7 +34787,7 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:K56"/>
-  <dataValidations count="3">
+  <dataValidations count="4">
     <dataValidation sqref="I2:I56" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"미지원,지원완료,서류합격,면접진행,최종합격,불합격"</formula1>
     </dataValidation>
@@ -34796,6 +34796,9 @@
     </dataValidation>
     <dataValidation sqref="B2:B56" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"AI_Agent_LLM,EEG_뇌공학_BCI,대기업_해외대,데이터사이언스,외국계금융_IB,전략컨설팅_RA"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D2:D56" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"1. 2026년 9월 마감 (긴급),2. 2026년 10월 마감 (긴급),3. 상시 / 즉시 지원 (ASAP),4. 2026년 12월 ~ 2027년 1월 (겨울 접수),5. 2027년 2~3월 (대기업 상반기),6. 2027년 3~4월 (현대차/연구실 사전컨택),7. 2027년 5월 (KAIST/IBS 하계인턴),8. 연중 수시 / 분기별 선발 (전략컨설팅 RA)"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
@@ -34869,15 +34872,15 @@
   <dimension ref="A1:I41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="44" customWidth="1" min="2" max="2"/>
     <col width="46" customWidth="1" min="3" max="3"/>
-    <col width="32" customWidth="1" min="4" max="4"/>
-    <col width="26" customWidth="1" min="5" max="5"/>
-    <col width="50" customWidth="1" min="6" max="6"/>
-    <col width="46" customWidth="1" min="7" max="7"/>
-    <col width="40" customWidth="1" min="8" max="8"/>
-    <col width="36" customWidth="1" min="9" max="9"/>
+    <col width="46" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="52" customWidth="1" min="6" max="6"/>
+    <col width="48" customWidth="1" min="7" max="7"/>
+    <col width="42" customWidth="1" min="8" max="8"/>
+    <col width="38" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -36554,6 +36557,11 @@
     <mergeCell ref="A18:I18"/>
     <mergeCell ref="A29:H29"/>
   </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="B3:B16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Data Analyst,Data Scientist,Business Analyst,Business / Ops Analyst"</formula1>
+    </dataValidation>
+  </dataValidations>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I3" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I4" r:id="rId2"/>
@@ -36603,15 +36611,15 @@
   <dimension ref="A1:I30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="36" customWidth="1" min="1" max="1"/>
-    <col width="44" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="36" customWidth="1" min="4" max="4"/>
-    <col width="50" customWidth="1" min="5" max="5"/>
-    <col width="50" customWidth="1" min="6" max="6"/>
-    <col width="50" customWidth="1" min="7" max="7"/>
-    <col width="40" customWidth="1" min="8" max="8"/>
-    <col width="36" customWidth="1" min="9" max="9"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="48" customWidth="1" min="2" max="2"/>
+    <col width="48" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
+    <col width="52" customWidth="1" min="5" max="5"/>
+    <col width="52" customWidth="1" min="6" max="6"/>
+    <col width="52" customWidth="1" min="7" max="7"/>
+    <col width="42" customWidth="1" min="8" max="8"/>
+    <col width="38" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -37757,6 +37765,11 @@
     <mergeCell ref="A23:I23"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="D3:D13" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"수시 채용,상시 채용,상시 수시 채용,연 1회 정기 공채,연 3회 정기 (봄/여름/겨울) &amp; 수시,매년 가을 공채 (페널티메이트)"</formula1>
+    </dataValidation>
+  </dataValidations>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H3" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H4" r:id="rId2"/>
@@ -37796,10 +37809,10 @@
   <dimension ref="A1:E29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="50" customWidth="1" min="1" max="1"/>
     <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="38" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="56" customWidth="1" min="3" max="3"/>
+    <col width="48" customWidth="1" min="4" max="4"/>
     <col width="26" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
@@ -38597,12 +38610,12 @@
   <dimension ref="A1:K85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="40" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="36" customWidth="1" min="5" max="5"/>
-    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="50" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="38" customWidth="1" min="5" max="5"/>
+    <col width="52" customWidth="1" min="6" max="6"/>
     <col hidden="1" width="13" customWidth="1" min="7" max="7"/>
     <col hidden="1" width="13" customWidth="1" min="8" max="8"/>
     <col hidden="1" width="13" customWidth="1" min="9" max="9"/>
@@ -41349,7 +41362,7 @@
       <c r="F85" s="124" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F85"/>
+  <autoFilter ref="A1:K85"/>
   <mergeCells count="56">
     <mergeCell ref="C56:C58"/>
     <mergeCell ref="A8:A10"/>
@@ -41408,6 +41421,11 @@
     <mergeCell ref="C71:C73"/>
     <mergeCell ref="A56:A58"/>
   </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="G2:G85" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"VERIFIED_VALID,PENDING,UNVERIFIED"</formula1>
+    </dataValidation>
+  </dataValidations>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId2"/>

</xml_diff>

<commit_message>
fix(ssot): restore shifted UK Top Targets hyperlinks, robustify expired date filtering, and add comprehensive edge-case tests
</commit_message>
<xml_diff>
--- a/Master_Internship_Tracker_2027_SSOT.xlsx
+++ b/Master_Internship_Tracker_2027_SSOT.xlsx
@@ -33,7 +33,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="34">
+  <fonts count="35">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -127,6 +127,12 @@
       <b val="1"/>
       <color rgb="001F4E79"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="000563C1"/>
+      <sz val="10"/>
+      <u val="single"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -534,7 +540,7 @@
     <xf numFmtId="0" fontId="13" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="16" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -555,7 +561,7 @@
     <xf numFmtId="0" fontId="13" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="16" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -576,7 +582,7 @@
     <xf numFmtId="0" fontId="13" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="16" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -588,10 +594,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -603,135 +609,135 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="19" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="22" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="19" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="21" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="15" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="26" fillId="15" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="16" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="29" fillId="16" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="16" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="16" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="27" fillId="16" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="17" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="28" fillId="16" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="17" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="17" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="17" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="28" fillId="17" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="18" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="29" fillId="18" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="18" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="18" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="28" fillId="18" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="19" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="29" fillId="19" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="19" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="19" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="28" fillId="19" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="20" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="29" fillId="20" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="20" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="20" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="28" fillId="20" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="22" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="30" fillId="22" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="23" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="29" fillId="23" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="23" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="32" fillId="23" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="23" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="23" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="33" fillId="23" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="28" fillId="24" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="29" fillId="24" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="24" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="32" fillId="24" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="24" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="34" fillId="24" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="23" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="33" fillId="24" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="23" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="27" fillId="23" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="24" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="23" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="24" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="27" fillId="24" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2884,8 +2890,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K15" r:id="rId14"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K16" r:id="rId15"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K17" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K19" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K20" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K20" r:id="rId19"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>